<commit_message>
v0.1: Added entity generator file (allowing x count of random entities to be made), then added to excel output file and constant .db file, executable dashboard run
</commit_message>
<xml_diff>
--- a/Source-files/Country_Codes_Scoring.xlsx
+++ b/Source-files/Country_Codes_Scoring.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\corru\PycharmProjects\Capital-Tracker\Source-files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4F043B08-00BC-4489-AE68-6469AF4E769E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D86EDCB-F1D4-4557-9BEB-05C3BA1C6DEC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2691,7 +2691,7 @@
     <col min="2" max="2" width="15.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="13.5703125" customWidth="1"/>
     <col min="4" max="4" width="12.5703125" customWidth="1"/>
-    <col min="5" max="5" width="13.42578125" customWidth="1"/>
+    <col min="5" max="5" width="13.42578125" hidden="1" customWidth="1"/>
     <col min="6" max="6" width="15.85546875" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>